<commit_message>
(stale commit 02/12) updated eval figures and files
</commit_message>
<xml_diff>
--- a/evals_20260214/0212_eval_log_jog.xlsx
+++ b/evals_20260214/0212_eval_log_jog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\findp\emphasis_markov\evals_20260214\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14243DDD-DD25-4B0A-B719-2E823F860595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8AFED70-C5A9-45A3-B6FB-11109E97AE72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="51">
   <si>
     <t>Unique Tags (%)</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>p &gt; 0.0083</t>
+  </si>
+  <si>
+    <t>Emphasis+Tags</t>
   </si>
 </sst>
 </file>
@@ -808,10 +811,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="14" width="13" customWidth="1"/>
+    <col min="1" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="4" max="14" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -827,7 +832,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -1523,20 +1528,20 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B22">
-        <f>AVERAGE(B6:B19)</f>
-        <v>162.85435217</v>
+        <f t="shared" ref="B22:D22" si="1">MEDIAN(B3:B20)</f>
+        <v>48.490165099999999</v>
       </c>
       <c r="C22">
-        <f t="shared" ref="C22:E22" si="1">AVERAGE(C6:C19)</f>
-        <v>183.29291471500002</v>
+        <f t="shared" si="1"/>
+        <v>63.030030019999998</v>
       </c>
       <c r="D22">
         <f t="shared" si="1"/>
-        <v>142.77051046142856</v>
+        <v>26.655578005000002</v>
       </c>
       <c r="E22">
-        <f t="shared" si="1"/>
-        <v>553.48156685071422</v>
+        <f>MEDIAN(E3:E20)</f>
+        <v>532.43013418999999</v>
       </c>
       <c r="H22" t="s">
         <v>47</v>
@@ -1567,6 +1572,22 @@
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <f>AVERAGE(B3:B20)</f>
+        <v>126.66449613222221</v>
+      </c>
+      <c r="C23">
+        <f>AVERAGE(C3:C20)</f>
+        <v>142.56115588944445</v>
+      </c>
+      <c r="D23">
+        <f>AVERAGE(D3:D20)</f>
+        <v>111.04373035888888</v>
+      </c>
+      <c r="E23">
+        <f>AVERAGE(E3:E20)</f>
+        <v>430.48566310611108</v>
+      </c>
       <c r="H23" t="s">
         <v>48</v>
       </c>
@@ -1947,6 +1968,24 @@
       </c>
       <c r="E44">
         <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B47">
+        <f>AVERAGE(B27:B44)</f>
+        <v>74.682648799944431</v>
+      </c>
+      <c r="C47">
+        <f t="shared" ref="C47:E47" si="5">AVERAGE(C27:C44)</f>
+        <v>62.720548746555565</v>
+      </c>
+      <c r="D47">
+        <f t="shared" si="5"/>
+        <v>135.71530548055554</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="5"/>
+        <v>283.78153237388892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>